<commit_message>
[fix]Fix error for load data
</commit_message>
<xml_diff>
--- a/data/data.xlsx
+++ b/data/data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jeong-uchan/Desktop/myLife/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64B3E642-EF4D-AE49-8CEC-12F679F988EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA37934F-B2CE-134A-B098-3509AB685733}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="740" windowWidth="30240" windowHeight="18900" xr2:uid="{D3448A19-EE9A-D84F-AF10-A95129378CE2}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17200" xr2:uid="{D3448A19-EE9A-D84F-AF10-A95129378CE2}"/>
   </bookViews>
   <sheets>
     <sheet name="2025" sheetId="1" r:id="rId1"/>
@@ -1000,9 +1000,6 @@
       <c r="A33" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="E33">
-        <v>67</v>
-      </c>
       <c r="G33"/>
     </row>
     <row r="34" spans="1:12">
@@ -1010,10 +1007,10 @@
         <v>54</v>
       </c>
       <c r="E34">
-        <v>70</v>
+        <v>100</v>
       </c>
       <c r="F34">
-        <v>48962</v>
+        <v>82640</v>
       </c>
       <c r="G34"/>
     </row>

</xml_diff>

<commit_message>
fix result tab error
</commit_message>
<xml_diff>
--- a/data/data.xlsx
+++ b/data/data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jeong-uchan/Desktop/myLife/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA37934F-B2CE-134A-B098-3509AB685733}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{709E5D6B-B2B6-A144-AAA0-B5008106E773}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17200" xr2:uid="{D3448A19-EE9A-D84F-AF10-A95129378CE2}"/>
+    <workbookView xWindow="2420" yWindow="760" windowWidth="30240" windowHeight="17200" xr2:uid="{D3448A19-EE9A-D84F-AF10-A95129378CE2}"/>
   </bookViews>
   <sheets>
     <sheet name="2025" sheetId="1" r:id="rId1"/>

</xml_diff>